<commit_message>
Curva S actualizada 2026-07-01 20:02 UTC
</commit_message>
<xml_diff>
--- a/data/50001544 - DMC MINING SERVICES.xlsx
+++ b/data/50001544 - DMC MINING SERVICES.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1525" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1525" uniqueCount="383">
   <si>
     <t xml:space="preserve"> 50001544 - DMC MINING SERVICES </t>
   </si>
@@ -1045,6 +1045,9 @@
   </si>
   <si>
     <t>1214909311722244</t>
+  </si>
+  <si>
+    <t>DESPACHADO Y FACTURADO</t>
   </si>
   <si>
     <t>Coordinacion Entrega con Cliente,OT 4313 - ZVN 1-9-45/2</t>
@@ -7734,7 +7737,7 @@
       </c>
       <c r="C103" s="9"/>
       <c r="D103" s="8">
-        <v>46197.49724334491</v>
+        <v>46204.802491932875</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>325</v>
@@ -7795,9 +7798,11 @@
       <c r="B104" s="5">
         <v>46160.65293966435</v>
       </c>
-      <c r="C104" s="6"/>
+      <c r="C104" s="5">
+        <v>46204.80222208334</v>
+      </c>
       <c r="D104" s="5">
-        <v>46197.60305672453</v>
+        <v>46204.80222355324</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>217</v>
@@ -7848,9 +7853,11 @@
       <c r="B105" s="8">
         <v>46160.652944201385</v>
       </c>
-      <c r="C105" s="9"/>
+      <c r="C105" s="8">
+        <v>46204.80248626157</v>
+      </c>
       <c r="D105" s="8">
-        <v>46197.49729465278</v>
+        <v>46204.80248778935</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>217</v>
@@ -7874,7 +7881,7 @@
         <v>26</v>
       </c>
       <c r="L105" s="9" t="s">
-        <v>26</v>
+        <v>332</v>
       </c>
       <c r="M105" s="9" t="s">
         <v>26</v>
@@ -7886,7 +7893,7 @@
         <v>217</v>
       </c>
       <c r="P105" s="9" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="Q105" s="9"/>
       <c r="R105" s="9"/>
@@ -7896,7 +7903,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B106" s="5">
         <v>46160.80816486111</v>
@@ -7906,7 +7913,7 @@
         <v>46160.817732083335</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7939,7 +7946,7 @@
         <v>58</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7949,7 +7956,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B107" s="8">
         <v>46160.80854525463</v>
@@ -7959,7 +7966,7 @@
         <v>46160.81773274306</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>26</v>
@@ -7992,7 +7999,7 @@
         <v>58</v>
       </c>
       <c r="P107" s="9" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="Q107" s="9"/>
       <c r="R107" s="9"/>
@@ -8002,7 +8009,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B108" s="5">
         <v>46160.65294850695</v>
@@ -8014,7 +8021,7 @@
         <v>46197.497765231485</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -8044,7 +8051,7 @@
         <v>322</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="P108" s="6" t="s">
         <v>322</v>
@@ -8067,7 +8074,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B109" s="8">
         <v>46160.652952592594</v>
@@ -8076,7 +8083,7 @@
         <v>46197.497369351855</v>
       </c>
       <c r="D109" s="8">
-        <v>46197.497371261576</v>
+        <v>46204.80222711805</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>217</v>
@@ -8106,13 +8113,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O109" s="9" t="s">
         <v>217</v>
       </c>
       <c r="P109" s="9" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Q109" s="9"/>
       <c r="R109" s="9"/>
@@ -8122,7 +8129,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B110" s="5">
         <v>46160.65295699074</v>
@@ -8131,7 +8138,7 @@
         <v>46197.497530023145</v>
       </c>
       <c r="D110" s="5">
-        <v>46197.49753173611</v>
+        <v>46204.80249248842</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>217</v>
@@ -8161,13 +8168,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>217</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -8177,7 +8184,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B111" s="8">
         <v>46160.809122164355</v>
@@ -8187,7 +8194,7 @@
         <v>46197.4977528125</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>26</v>
@@ -8214,13 +8221,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q111" s="9"/>
       <c r="R111" s="9"/>
@@ -8230,7 +8237,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B112" s="5">
         <v>46160.809137627315</v>
@@ -8240,7 +8247,7 @@
         <v>46197.497759895836</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8267,13 +8274,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8283,7 +8290,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B113" s="8">
         <v>46160.652961203705</v>
@@ -8293,7 +8300,7 @@
         <v>46194.05666876158</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>26</v>
@@ -8323,7 +8330,7 @@
         <v>322</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="P113" s="9" t="s">
         <v>322</v>
@@ -8346,7 +8353,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B114" s="5">
         <v>46160.65296532407</v>
@@ -8381,13 +8388,13 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O114" s="6" t="s">
         <v>217</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Q114" s="6"/>
       <c r="R114" s="6"/>
@@ -8397,7 +8404,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B115" s="8">
         <v>46160.65297267361</v>
@@ -8432,13 +8439,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O115" s="9" t="s">
         <v>217</v>
       </c>
       <c r="P115" s="9" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Q115" s="9"/>
       <c r="R115" s="9"/>
@@ -8448,7 +8455,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B116" s="5">
         <v>46160.81088733797</v>
@@ -8458,7 +8465,7 @@
         <v>46197.49775597222</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8483,13 +8490,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8499,7 +8506,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B117" s="8">
         <v>46160.81089606481</v>
@@ -8509,7 +8516,7 @@
         <v>46197.49776570602</v>
       </c>
       <c r="E117" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>26</v>
@@ -8534,13 +8541,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O117" s="9" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="P117" s="9" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q117" s="9"/>
       <c r="R117" s="9"/>
@@ -8550,7 +8557,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B118" s="5">
         <v>46160.65297846065</v>
@@ -8560,7 +8567,7 @@
         <v>46183.89564782407</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8590,10 +8597,10 @@
         <v>322</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Q118" s="5">
         <v>46217</v>
@@ -8613,7 +8620,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B119" s="8">
         <v>46160.652983935186</v>
@@ -8650,13 +8657,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O119" s="9" t="s">
         <v>217</v>
       </c>
       <c r="P119" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q119" s="9"/>
       <c r="R119" s="9"/>
@@ -8666,7 +8673,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B120" s="5">
         <v>46160.65298813657</v>
@@ -8703,13 +8710,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>217</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8719,7 +8726,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B121" s="8">
         <v>46160.81215837963</v>
@@ -8729,7 +8736,7 @@
         <v>46194.05454575231</v>
       </c>
       <c r="E121" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>26</v>
@@ -8756,13 +8763,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O121" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P121" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q121" s="9"/>
       <c r="R121" s="9"/>
@@ -8772,7 +8779,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B122" s="5">
         <v>46160.81220768519</v>
@@ -8782,7 +8789,7 @@
         <v>46194.05454428241</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
@@ -8809,13 +8816,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O122" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8825,7 +8832,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B123" s="8">
         <v>46160.65302554399</v>
@@ -8835,7 +8842,7 @@
         <v>46160.8192895949</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>25</v>
@@ -8859,7 +8866,7 @@
         <v>26</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P123" s="9" t="s">
         <v>26</v>
@@ -8872,7 +8879,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B124" s="5">
         <v>46160.65302895833</v>
@@ -8882,16 +8889,16 @@
         <v>46160.819199722224</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I124" s="5">
         <v>46218</v>
@@ -8909,13 +8916,13 @@
         <v>26</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q124" s="5">
         <v>46218</v>
@@ -8935,7 +8942,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B125" s="8">
         <v>46160.65303386574</v>
@@ -8945,7 +8952,7 @@
         <v>46199.75068079861</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>26</v>
@@ -8972,13 +8979,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O125" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="P125" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q125" s="8">
         <v>46218</v>
@@ -8998,7 +9005,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B126" s="5">
         <v>46160.65808951389</v>
@@ -9008,7 +9015,7 @@
         <v>46160.819809513894</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>25</v>
@@ -9032,7 +9039,7 @@
         <v>26</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P126" s="6" t="s">
         <v>26</v>
@@ -9051,7 +9058,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B127" s="8">
         <v>46160.66095159722</v>
@@ -9061,7 +9068,7 @@
         <v>46160.81972457176</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>26</v>
@@ -9088,13 +9095,13 @@
         <v>26</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O127" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="P127" s="9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="Q127" s="8">
         <v>46218</v>
@@ -9114,7 +9121,7 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B128" s="5">
         <v>46160.66107538194</v>
@@ -9124,7 +9131,7 @@
         <v>46160.8199466088</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
@@ -9151,13 +9158,13 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="Q128" s="5">
         <v>46227</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-22 13:49 UTC
</commit_message>
<xml_diff>
--- a/data/50001544 - DMC MINING SERVICES.xlsx
+++ b/data/50001544 - DMC MINING SERVICES.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1525" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="384">
   <si>
     <t xml:space="preserve"> 50001544 - DMC MINING SERVICES </t>
   </si>
@@ -1082,6 +1082,9 @@
   </si>
   <si>
     <t>Coordinacion Entrega con Cliente,OT 4314 - VDF VLT  FC 102</t>
+  </si>
+  <si>
+    <t>1216786101186166</t>
   </si>
   <si>
     <t>1214889077215248</t>
@@ -1746,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U128"/>
+  <dimension ref="A1:U129"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -7766,7 +7769,7 @@
       </c>
       <c r="C103" s="9"/>
       <c r="D103" s="8">
-        <v>46224.79338295139</v>
+        <v>46225.55379075231</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>324</v>
@@ -7937,9 +7940,11 @@
       <c r="B106" s="5">
         <v>46160.80816486111</v>
       </c>
-      <c r="C106" s="6"/>
+      <c r="C106" s="5">
+        <v>46225.55378449074</v>
+      </c>
       <c r="D106" s="5">
-        <v>46224.793388101854</v>
+        <v>46225.55378673611</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>334</v>
@@ -7988,47 +7993,41 @@
         <v>336</v>
       </c>
       <c r="B107" s="8">
-        <v>46160.80854525463</v>
+        <v>46225.55376708333</v>
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="8">
-        <v>46224.79338983796</v>
+        <v>46225.553774409724</v>
       </c>
       <c r="E107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H107" s="9"/>
+      <c r="I107" s="9"/>
+      <c r="J107" s="9"/>
+      <c r="K107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M107" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N107" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="F107" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G107" s="9" t="s">
-        <v>325</v>
-      </c>
-      <c r="H107" s="9" t="s">
-        <v>326</v>
-      </c>
-      <c r="I107" s="8">
-        <v>46212</v>
-      </c>
-      <c r="J107" s="8">
-        <v>46212</v>
-      </c>
-      <c r="K107" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L107" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M107" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N107" s="9" t="s">
-        <v>324</v>
-      </c>
       <c r="O107" s="9" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="P107" s="9" t="s">
-        <v>337</v>
+        <v>26</v>
       </c>
       <c r="Q107" s="9"/>
       <c r="R107" s="9"/>
@@ -8038,84 +8037,72 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="B108" s="5">
+        <v>46160.80854525463</v>
+      </c>
+      <c r="C108" s="6"/>
+      <c r="D108" s="5">
+        <v>46224.79338983796</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G108" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="I108" s="5">
+        <v>46212</v>
+      </c>
+      <c r="J108" s="5">
+        <v>46212</v>
+      </c>
+      <c r="K108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M108" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N108" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="O108" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="P108" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="B108" s="5">
-        <v>46160.65294850695</v>
-      </c>
-      <c r="C108" s="5">
-        <v>46197.49765626158</v>
-      </c>
-      <c r="D108" s="5">
-        <v>46223.58126640046</v>
-      </c>
-      <c r="E108" s="6" t="s">
-        <v>339</v>
-      </c>
-      <c r="F108" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G108" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="H108" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I108" s="5">
-        <v>46213</v>
-      </c>
-      <c r="J108" s="5">
-        <v>46213</v>
-      </c>
-      <c r="K108" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L108" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M108" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N108" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="O108" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="P108" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="Q108" s="5">
-        <v>46213</v>
-      </c>
-      <c r="R108" s="5">
-        <v>46213</v>
-      </c>
-      <c r="S108" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T108" s="6">
-        <v>1</v>
-      </c>
-      <c r="U108" s="12" t="s">
-        <v>68</v>
-      </c>
+      <c r="Q108" s="6"/>
+      <c r="R108" s="6"/>
+      <c r="S108" s="6"/>
+      <c r="T108" s="6"/>
+      <c r="U108" s="6"/>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B109" s="8">
-        <v>46160.652952592594</v>
+        <v>46160.65294850695</v>
       </c>
       <c r="C109" s="8">
-        <v>46197.497369351855</v>
+        <v>46197.49765626158</v>
       </c>
       <c r="D109" s="8">
-        <v>46223.58121423611</v>
+        <v>46223.58126640046</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>216</v>
+        <v>340</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>26</v>
@@ -8142,32 +8129,42 @@
         <v>26</v>
       </c>
       <c r="N109" s="9" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="O109" s="9" t="s">
-        <v>216</v>
+        <v>341</v>
       </c>
       <c r="P109" s="9" t="s">
-        <v>342</v>
-      </c>
-      <c r="Q109" s="9"/>
-      <c r="R109" s="9"/>
-      <c r="S109" s="9"/>
-      <c r="T109" s="9"/>
-      <c r="U109" s="9"/>
+        <v>321</v>
+      </c>
+      <c r="Q109" s="8">
+        <v>46213</v>
+      </c>
+      <c r="R109" s="8">
+        <v>46213</v>
+      </c>
+      <c r="S109" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T109" s="9">
+        <v>1</v>
+      </c>
+      <c r="U109" s="12" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B110" s="5">
-        <v>46160.65295699074</v>
+        <v>46160.652952592594</v>
       </c>
       <c r="C110" s="5">
-        <v>46197.497530023145</v>
+        <v>46197.497369351855</v>
       </c>
       <c r="D110" s="5">
-        <v>46223.581210069446</v>
+        <v>46223.58121423611</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>216</v>
@@ -8197,13 +8194,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>216</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -8216,14 +8213,16 @@
         <v>344</v>
       </c>
       <c r="B111" s="8">
-        <v>46160.809122164355</v>
-      </c>
-      <c r="C111" s="9"/>
+        <v>46160.65295699074</v>
+      </c>
+      <c r="C111" s="8">
+        <v>46197.497530023145</v>
+      </c>
       <c r="D111" s="8">
-        <v>46223.58120212963</v>
+        <v>46223.581210069446</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>26</v>
@@ -8250,13 +8249,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="Q111" s="9"/>
       <c r="R111" s="9"/>
@@ -8266,17 +8265,17 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B112" s="5">
-        <v>46160.809137627315</v>
+        <v>46160.809122164355</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46223.58120152778</v>
+        <v>46225.55379164351</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8303,13 +8302,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O112" s="6" t="s">
         <v>334</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8319,32 +8318,32 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B113" s="8">
-        <v>46160.652961203705</v>
+        <v>46160.809137627315</v>
       </c>
       <c r="C113" s="9"/>
       <c r="D113" s="8">
-        <v>46217.178433506946</v>
+        <v>46223.58120152778</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G113" s="9" t="s">
-        <v>246</v>
+        <v>91</v>
       </c>
       <c r="H113" s="9" t="s">
-        <v>247</v>
+        <v>91</v>
       </c>
       <c r="I113" s="8">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="J113" s="8">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="K113" s="9" t="s">
         <v>26</v>
@@ -8356,43 +8355,33 @@
         <v>26</v>
       </c>
       <c r="N113" s="9" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="P113" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="Q113" s="8">
-        <v>46216</v>
-      </c>
-      <c r="R113" s="8">
-        <v>46216</v>
-      </c>
-      <c r="S113" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T113" s="9">
-        <v>1</v>
-      </c>
-      <c r="U113" s="10" t="s">
-        <v>33</v>
-      </c>
+        <v>346</v>
+      </c>
+      <c r="Q113" s="9"/>
+      <c r="R113" s="9"/>
+      <c r="S113" s="9"/>
+      <c r="T113" s="9"/>
+      <c r="U113" s="9"/>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B114" s="5">
-        <v>46160.65296532407</v>
+        <v>46160.652961203705</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46216.168960752315</v>
+        <v>46217.178433506946</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>216</v>
+        <v>350</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
@@ -8403,7 +8392,9 @@
       <c r="H114" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I114" s="6"/>
+      <c r="I114" s="5">
+        <v>46216</v>
+      </c>
       <c r="J114" s="5">
         <v>46216</v>
       </c>
@@ -8417,30 +8408,40 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>349</v>
+        <v>321</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>216</v>
+        <v>351</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>352</v>
-      </c>
-      <c r="Q114" s="6"/>
-      <c r="R114" s="6"/>
-      <c r="S114" s="6"/>
-      <c r="T114" s="6"/>
-      <c r="U114" s="6"/>
+        <v>321</v>
+      </c>
+      <c r="Q114" s="5">
+        <v>46216</v>
+      </c>
+      <c r="R114" s="5">
+        <v>46216</v>
+      </c>
+      <c r="S114" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T114" s="6">
+        <v>1</v>
+      </c>
+      <c r="U114" s="10" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B115" s="8">
-        <v>46160.65297267361</v>
+        <v>46160.65296532407</v>
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46216.16895939814</v>
+        <v>46216.168960752315</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>216</v>
@@ -8468,13 +8469,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O115" s="9" t="s">
         <v>216</v>
       </c>
       <c r="P115" s="9" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="Q115" s="9"/>
       <c r="R115" s="9"/>
@@ -8484,17 +8485,17 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B116" s="5">
-        <v>46160.81088733797</v>
+        <v>46160.65297267361</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46216.16896737269</v>
+        <v>46216.16895939814</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8519,13 +8520,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8535,14 +8536,14 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B117" s="8">
-        <v>46160.81089606481</v>
+        <v>46160.81088733797</v>
       </c>
       <c r="C117" s="9"/>
       <c r="D117" s="8">
-        <v>46216.168969085644</v>
+        <v>46216.16896737269</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>334</v>
@@ -8570,13 +8571,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O117" s="9" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="P117" s="9" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q117" s="9"/>
       <c r="R117" s="9"/>
@@ -8589,14 +8590,14 @@
         <v>358</v>
       </c>
       <c r="B118" s="5">
-        <v>46160.65297846065</v>
+        <v>46160.81089606481</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46218.17912671296</v>
+        <v>46216.168969085644</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>359</v>
+        <v>334</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8607,11 +8608,9 @@
       <c r="H118" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I118" s="5">
-        <v>46217</v>
-      </c>
+      <c r="I118" s="6"/>
       <c r="J118" s="5">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="K118" s="6" t="s">
         <v>26</v>
@@ -8623,43 +8622,33 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>321</v>
+        <v>350</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="Q118" s="5">
-        <v>46217</v>
-      </c>
-      <c r="R118" s="5">
-        <v>46217</v>
-      </c>
-      <c r="S118" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T118" s="6">
-        <v>0</v>
-      </c>
-      <c r="U118" s="11" t="s">
-        <v>120</v>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="Q118" s="6"/>
+      <c r="R118" s="6"/>
+      <c r="S118" s="6"/>
+      <c r="T118" s="6"/>
+      <c r="U118" s="6"/>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B119" s="8">
-        <v>46160.652983935186</v>
+        <v>46160.65297846065</v>
       </c>
       <c r="C119" s="9"/>
       <c r="D119" s="8">
-        <v>46217.16843326389</v>
+        <v>46218.17912671296</v>
       </c>
       <c r="E119" s="9" t="s">
-        <v>216</v>
+        <v>360</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>26</v>
@@ -8686,30 +8675,40 @@
         <v>26</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>359</v>
+        <v>321</v>
       </c>
       <c r="O119" s="9" t="s">
-        <v>216</v>
+        <v>351</v>
       </c>
       <c r="P119" s="9" t="s">
-        <v>359</v>
-      </c>
-      <c r="Q119" s="9"/>
-      <c r="R119" s="9"/>
-      <c r="S119" s="9"/>
-      <c r="T119" s="9"/>
-      <c r="U119" s="9"/>
+        <v>361</v>
+      </c>
+      <c r="Q119" s="8">
+        <v>46217</v>
+      </c>
+      <c r="R119" s="8">
+        <v>46217</v>
+      </c>
+      <c r="S119" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T119" s="9">
+        <v>0</v>
+      </c>
+      <c r="U119" s="11" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>362</v>
       </c>
       <c r="B120" s="5">
-        <v>46160.65298813657</v>
+        <v>46160.652983935186</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46217.16837645833</v>
+        <v>46217.16843326389</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>216</v>
@@ -8739,13 +8738,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>216</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8758,14 +8757,14 @@
         <v>363</v>
       </c>
       <c r="B121" s="8">
-        <v>46160.81215837963</v>
+        <v>46160.65298813657</v>
       </c>
       <c r="C121" s="9"/>
       <c r="D121" s="8">
-        <v>46217.168417002315</v>
+        <v>46217.16837645833</v>
       </c>
       <c r="E121" s="9" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>26</v>
@@ -8792,13 +8791,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O121" s="9" t="s">
-        <v>334</v>
+        <v>216</v>
       </c>
       <c r="P121" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q121" s="9"/>
       <c r="R121" s="9"/>
@@ -8811,11 +8810,11 @@
         <v>364</v>
       </c>
       <c r="B122" s="5">
-        <v>46160.81220768519</v>
+        <v>46160.81215837963</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46217.16841864583</v>
+        <v>46217.168417002315</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>334</v>
@@ -8845,13 +8844,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>334</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8864,24 +8863,30 @@
         <v>365</v>
       </c>
       <c r="B123" s="8">
-        <v>46160.65302554399</v>
+        <v>46160.81220768519</v>
       </c>
       <c r="C123" s="9"/>
       <c r="D123" s="8">
-        <v>46160.8192895949</v>
+        <v>46217.16841864583</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>366</v>
+        <v>334</v>
       </c>
       <c r="F123" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G123" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H123" s="9"/>
-      <c r="I123" s="9"/>
-      <c r="J123" s="9"/>
+        <v>246</v>
+      </c>
+      <c r="H123" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="I123" s="8">
+        <v>46217</v>
+      </c>
+      <c r="J123" s="8">
+        <v>46217</v>
+      </c>
       <c r="K123" s="9" t="s">
         <v>26</v>
       </c>
@@ -8889,16 +8894,16 @@
         <v>26</v>
       </c>
       <c r="M123" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>26</v>
+        <v>360</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>367</v>
+        <v>334</v>
       </c>
       <c r="P123" s="9" t="s">
-        <v>26</v>
+        <v>360</v>
       </c>
       <c r="Q123" s="9"/>
       <c r="R123" s="9"/>
@@ -8908,33 +8913,27 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B124" s="5">
-        <v>46160.65302895833</v>
+        <v>46160.65302554399</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46219.173083553236</v>
+        <v>46160.8192895949</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="H124" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="I124" s="5">
-        <v>46218</v>
-      </c>
-      <c r="J124" s="5">
-        <v>46226</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H124" s="6"/>
+      <c r="I124" s="6"/>
+      <c r="J124" s="6"/>
       <c r="K124" s="6" t="s">
         <v>26</v>
       </c>
@@ -8942,55 +8941,45 @@
         <v>26</v>
       </c>
       <c r="M124" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>366</v>
+        <v>26</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>366</v>
-      </c>
-      <c r="Q124" s="5">
-        <v>46218</v>
-      </c>
-      <c r="R124" s="5">
-        <v>46226</v>
-      </c>
-      <c r="S124" s="12" t="s">
-        <v>372</v>
-      </c>
-      <c r="T124" s="6">
-        <v>0</v>
-      </c>
-      <c r="U124" s="11" t="s">
-        <v>120</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q124" s="6"/>
+      <c r="R124" s="6"/>
+      <c r="S124" s="6"/>
+      <c r="T124" s="6"/>
+      <c r="U124" s="6"/>
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B125" s="8">
-        <v>46160.65303386574</v>
+        <v>46160.65302895833</v>
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="8">
-        <v>46219.17308424768</v>
+        <v>46219.173083553236</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>36</v>
+        <v>371</v>
       </c>
       <c r="H125" s="9" t="s">
-        <v>37</v>
+        <v>372</v>
       </c>
       <c r="I125" s="8">
         <v>46218</v>
@@ -9008,13 +8997,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O125" s="9" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="P125" s="9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="Q125" s="8">
         <v>46218</v>
@@ -9023,7 +9012,7 @@
         <v>46226</v>
       </c>
       <c r="S125" s="12" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="T125" s="9">
         <v>0</v>
@@ -9034,27 +9023,33 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B126" s="5">
-        <v>46160.65808951389</v>
+        <v>46160.65303386574</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46160.819809513894</v>
+        <v>46219.17308424768</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H126" s="6"/>
-      <c r="I126" s="6"/>
-      <c r="J126" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="H126" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I126" s="5">
+        <v>46218</v>
+      </c>
+      <c r="J126" s="5">
+        <v>46226</v>
+      </c>
       <c r="K126" s="6" t="s">
         <v>26</v>
       </c>
@@ -9062,21 +9057,25 @@
         <v>26</v>
       </c>
       <c r="M126" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>26</v>
+        <v>367</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>377</v>
+        <v>360</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q126" s="6"/>
-      <c r="R126" s="6"/>
-      <c r="S126" s="10" t="s">
-        <v>32</v>
+        <v>367</v>
+      </c>
+      <c r="Q126" s="5">
+        <v>46218</v>
+      </c>
+      <c r="R126" s="5">
+        <v>46226</v>
+      </c>
+      <c r="S126" s="12" t="s">
+        <v>373</v>
       </c>
       <c r="T126" s="6">
         <v>0</v>
@@ -9087,33 +9086,27 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B127" s="8">
-        <v>46160.66095159722</v>
+        <v>46160.65808951389</v>
       </c>
       <c r="C127" s="9"/>
       <c r="D127" s="8">
-        <v>46219.173089097225</v>
+        <v>46160.819809513894</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F127" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G127" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="H127" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I127" s="8">
-        <v>46218</v>
-      </c>
-      <c r="J127" s="8">
-        <v>46226</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H127" s="9"/>
+      <c r="I127" s="9"/>
+      <c r="J127" s="9"/>
       <c r="K127" s="9" t="s">
         <v>26</v>
       </c>
@@ -9121,25 +9114,21 @@
         <v>26</v>
       </c>
       <c r="M127" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>376</v>
+        <v>26</v>
       </c>
       <c r="O127" s="9" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="P127" s="9" t="s">
-        <v>380</v>
-      </c>
-      <c r="Q127" s="8">
-        <v>46218</v>
-      </c>
-      <c r="R127" s="8">
-        <v>46226</v>
-      </c>
-      <c r="S127" s="12" t="s">
-        <v>372</v>
+        <v>26</v>
+      </c>
+      <c r="Q127" s="9"/>
+      <c r="R127" s="9"/>
+      <c r="S127" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T127" s="9">
         <v>0</v>
@@ -9150,17 +9139,17 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B128" s="5">
-        <v>46160.66107538194</v>
+        <v>46160.66095159722</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46160.8199466088</v>
+        <v>46219.173089097225</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
@@ -9172,10 +9161,10 @@
         <v>55</v>
       </c>
       <c r="I128" s="5">
-        <v>46227</v>
+        <v>46218</v>
       </c>
       <c r="J128" s="5">
-        <v>46237</v>
+        <v>46226</v>
       </c>
       <c r="K128" s="6" t="s">
         <v>26</v>
@@ -9187,27 +9176,90 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>379</v>
+        <v>360</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="Q128" s="5">
-        <v>46227</v>
+        <v>46218</v>
       </c>
       <c r="R128" s="5">
-        <v>46237</v>
-      </c>
-      <c r="S128" s="10" t="s">
-        <v>32</v>
+        <v>46226</v>
+      </c>
+      <c r="S128" s="12" t="s">
+        <v>373</v>
       </c>
       <c r="T128" s="6">
         <v>0</v>
       </c>
       <c r="U128" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="129" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A129" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="B129" s="8">
+        <v>46160.66107538194</v>
+      </c>
+      <c r="C129" s="9"/>
+      <c r="D129" s="8">
+        <v>46160.8199466088</v>
+      </c>
+      <c r="E129" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="F129" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G129" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="H129" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="I129" s="8">
+        <v>46227</v>
+      </c>
+      <c r="J129" s="8">
+        <v>46237</v>
+      </c>
+      <c r="K129" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L129" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M129" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N129" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="O129" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="P129" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="Q129" s="8">
+        <v>46227</v>
+      </c>
+      <c r="R129" s="8">
+        <v>46237</v>
+      </c>
+      <c r="S129" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="T129" s="9">
+        <v>0</v>
+      </c>
+      <c r="U129" s="11" t="s">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-22 16:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001544 - DMC MINING SERVICES.xlsx
+++ b/data/50001544 - DMC MINING SERVICES.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1525" uniqueCount="383">
   <si>
     <t xml:space="preserve"> 50001544 - DMC MINING SERVICES </t>
   </si>
@@ -1082,9 +1082,6 @@
   </si>
   <si>
     <t>Coordinacion Entrega con Cliente,OT 4314 - VDF VLT  FC 102</t>
-  </si>
-  <si>
-    <t>1216786101186166</t>
   </si>
   <si>
     <t>1214889077215248</t>
@@ -1749,7 +1746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U129"/>
+  <dimension ref="A1:U128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -7993,24 +7990,30 @@
         <v>336</v>
       </c>
       <c r="B107" s="8">
-        <v>46225.55376708333</v>
+        <v>46160.80854525463</v>
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="8">
-        <v>46225.553774409724</v>
+        <v>46224.79338983796</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>26</v>
+        <v>334</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G107" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H107" s="9"/>
-      <c r="I107" s="9"/>
-      <c r="J107" s="9"/>
+        <v>325</v>
+      </c>
+      <c r="H107" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="I107" s="8">
+        <v>46212</v>
+      </c>
+      <c r="J107" s="8">
+        <v>46212</v>
+      </c>
       <c r="K107" s="9" t="s">
         <v>26</v>
       </c>
@@ -8021,13 +8024,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="9" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="O107" s="9" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="P107" s="9" t="s">
-        <v>26</v>
+        <v>337</v>
       </c>
       <c r="Q107" s="9"/>
       <c r="R107" s="9"/>
@@ -8037,32 +8040,34 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B108" s="5">
-        <v>46160.80854525463</v>
-      </c>
-      <c r="C108" s="6"/>
+        <v>46160.65294850695</v>
+      </c>
+      <c r="C108" s="5">
+        <v>46197.49765626158</v>
+      </c>
       <c r="D108" s="5">
-        <v>46224.79338983796</v>
+        <v>46223.58126640046</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>325</v>
+        <v>91</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>326</v>
+        <v>91</v>
       </c>
       <c r="I108" s="5">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="J108" s="5">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="K108" s="6" t="s">
         <v>26</v>
@@ -8074,35 +8079,45 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>58</v>
+        <v>340</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="Q108" s="6"/>
-      <c r="R108" s="6"/>
-      <c r="S108" s="6"/>
-      <c r="T108" s="6"/>
-      <c r="U108" s="6"/>
+        <v>321</v>
+      </c>
+      <c r="Q108" s="5">
+        <v>46213</v>
+      </c>
+      <c r="R108" s="5">
+        <v>46213</v>
+      </c>
+      <c r="S108" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T108" s="6">
+        <v>1</v>
+      </c>
+      <c r="U108" s="12" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B109" s="8">
-        <v>46160.65294850695</v>
+        <v>46160.652952592594</v>
       </c>
       <c r="C109" s="8">
-        <v>46197.49765626158</v>
+        <v>46197.497369351855</v>
       </c>
       <c r="D109" s="8">
-        <v>46223.58126640046</v>
+        <v>46223.58121423611</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>340</v>
+        <v>216</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>26</v>
@@ -8129,42 +8144,32 @@
         <v>26</v>
       </c>
       <c r="N109" s="9" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="O109" s="9" t="s">
-        <v>341</v>
+        <v>216</v>
       </c>
       <c r="P109" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="Q109" s="8">
-        <v>46213</v>
-      </c>
-      <c r="R109" s="8">
-        <v>46213</v>
-      </c>
-      <c r="S109" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T109" s="9">
-        <v>1</v>
-      </c>
-      <c r="U109" s="12" t="s">
-        <v>68</v>
-      </c>
+        <v>342</v>
+      </c>
+      <c r="Q109" s="9"/>
+      <c r="R109" s="9"/>
+      <c r="S109" s="9"/>
+      <c r="T109" s="9"/>
+      <c r="U109" s="9"/>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B110" s="5">
-        <v>46160.652952592594</v>
+        <v>46160.65295699074</v>
       </c>
       <c r="C110" s="5">
-        <v>46197.497369351855</v>
+        <v>46197.497530023145</v>
       </c>
       <c r="D110" s="5">
-        <v>46223.58121423611</v>
+        <v>46223.581210069446</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>216</v>
@@ -8194,13 +8199,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>216</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -8213,16 +8218,14 @@
         <v>344</v>
       </c>
       <c r="B111" s="8">
-        <v>46160.65295699074</v>
-      </c>
-      <c r="C111" s="8">
-        <v>46197.497530023145</v>
-      </c>
+        <v>46160.809122164355</v>
+      </c>
+      <c r="C111" s="9"/>
       <c r="D111" s="8">
-        <v>46223.581210069446</v>
+        <v>46225.55379164351</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>26</v>
@@ -8249,13 +8252,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="Q111" s="9"/>
       <c r="R111" s="9"/>
@@ -8265,17 +8268,17 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B112" s="5">
-        <v>46160.809122164355</v>
+        <v>46160.809137627315</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46225.55379164351</v>
+        <v>46223.58120152778</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8302,13 +8305,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="O112" s="6" t="s">
         <v>334</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8318,32 +8321,32 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B113" s="8">
-        <v>46160.809137627315</v>
+        <v>46160.652961203705</v>
       </c>
       <c r="C113" s="9"/>
       <c r="D113" s="8">
-        <v>46223.58120152778</v>
+        <v>46217.178433506946</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G113" s="9" t="s">
-        <v>91</v>
+        <v>246</v>
       </c>
       <c r="H113" s="9" t="s">
-        <v>91</v>
+        <v>247</v>
       </c>
       <c r="I113" s="8">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="J113" s="8">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="K113" s="9" t="s">
         <v>26</v>
@@ -8355,33 +8358,43 @@
         <v>26</v>
       </c>
       <c r="N113" s="9" t="s">
-        <v>340</v>
+        <v>321</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="P113" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="Q113" s="9"/>
-      <c r="R113" s="9"/>
-      <c r="S113" s="9"/>
-      <c r="T113" s="9"/>
-      <c r="U113" s="9"/>
+        <v>321</v>
+      </c>
+      <c r="Q113" s="8">
+        <v>46216</v>
+      </c>
+      <c r="R113" s="8">
+        <v>46216</v>
+      </c>
+      <c r="S113" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T113" s="9">
+        <v>1</v>
+      </c>
+      <c r="U113" s="10" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B114" s="5">
-        <v>46160.652961203705</v>
+        <v>46160.65296532407</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46217.178433506946</v>
+        <v>46216.168960752315</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>350</v>
+        <v>216</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
@@ -8392,9 +8405,7 @@
       <c r="H114" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I114" s="5">
-        <v>46216</v>
-      </c>
+      <c r="I114" s="6"/>
       <c r="J114" s="5">
         <v>46216</v>
       </c>
@@ -8408,40 +8419,30 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>321</v>
+        <v>349</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>351</v>
+        <v>216</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="Q114" s="5">
-        <v>46216</v>
-      </c>
-      <c r="R114" s="5">
-        <v>46216</v>
-      </c>
-      <c r="S114" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T114" s="6">
-        <v>1</v>
-      </c>
-      <c r="U114" s="10" t="s">
-        <v>33</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="Q114" s="6"/>
+      <c r="R114" s="6"/>
+      <c r="S114" s="6"/>
+      <c r="T114" s="6"/>
+      <c r="U114" s="6"/>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B115" s="8">
-        <v>46160.65296532407</v>
+        <v>46160.65297267361</v>
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46216.168960752315</v>
+        <v>46216.16895939814</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>216</v>
@@ -8469,13 +8470,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="O115" s="9" t="s">
         <v>216</v>
       </c>
       <c r="P115" s="9" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="Q115" s="9"/>
       <c r="R115" s="9"/>
@@ -8485,17 +8486,17 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B116" s="5">
-        <v>46160.65297267361</v>
+        <v>46160.81088733797</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46216.16895939814</v>
+        <v>46216.16896737269</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8520,13 +8521,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8536,14 +8537,14 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B117" s="8">
-        <v>46160.81088733797</v>
+        <v>46160.81089606481</v>
       </c>
       <c r="C117" s="9"/>
       <c r="D117" s="8">
-        <v>46216.16896737269</v>
+        <v>46216.168969085644</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>334</v>
@@ -8571,13 +8572,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="O117" s="9" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="P117" s="9" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="Q117" s="9"/>
       <c r="R117" s="9"/>
@@ -8590,14 +8591,14 @@
         <v>358</v>
       </c>
       <c r="B118" s="5">
-        <v>46160.81089606481</v>
+        <v>46160.65297846065</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46216.168969085644</v>
+        <v>46218.17912671296</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>334</v>
+        <v>359</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8608,9 +8609,11 @@
       <c r="H118" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I118" s="6"/>
+      <c r="I118" s="5">
+        <v>46217</v>
+      </c>
       <c r="J118" s="5">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="K118" s="6" t="s">
         <v>26</v>
@@ -8622,33 +8625,43 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="O118" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="O118" s="6" t="s">
-        <v>348</v>
-      </c>
       <c r="P118" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="Q118" s="6"/>
-      <c r="R118" s="6"/>
-      <c r="S118" s="6"/>
-      <c r="T118" s="6"/>
-      <c r="U118" s="6"/>
+        <v>360</v>
+      </c>
+      <c r="Q118" s="5">
+        <v>46217</v>
+      </c>
+      <c r="R118" s="5">
+        <v>46217</v>
+      </c>
+      <c r="S118" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="T118" s="6">
+        <v>0</v>
+      </c>
+      <c r="U118" s="11" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B119" s="8">
-        <v>46160.65297846065</v>
+        <v>46160.652983935186</v>
       </c>
       <c r="C119" s="9"/>
       <c r="D119" s="8">
-        <v>46218.17912671296</v>
+        <v>46217.16843326389</v>
       </c>
       <c r="E119" s="9" t="s">
-        <v>360</v>
+        <v>216</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>26</v>
@@ -8675,40 +8688,30 @@
         <v>26</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>321</v>
+        <v>359</v>
       </c>
       <c r="O119" s="9" t="s">
-        <v>351</v>
+        <v>216</v>
       </c>
       <c r="P119" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="Q119" s="8">
-        <v>46217</v>
-      </c>
-      <c r="R119" s="8">
-        <v>46217</v>
-      </c>
-      <c r="S119" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="T119" s="9">
-        <v>0</v>
-      </c>
-      <c r="U119" s="11" t="s">
-        <v>120</v>
-      </c>
+        <v>359</v>
+      </c>
+      <c r="Q119" s="9"/>
+      <c r="R119" s="9"/>
+      <c r="S119" s="9"/>
+      <c r="T119" s="9"/>
+      <c r="U119" s="9"/>
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
         <v>362</v>
       </c>
       <c r="B120" s="5">
-        <v>46160.652983935186</v>
+        <v>46160.65298813657</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46217.16843326389</v>
+        <v>46217.16837645833</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>216</v>
@@ -8738,13 +8741,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>216</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8757,14 +8760,14 @@
         <v>363</v>
       </c>
       <c r="B121" s="8">
-        <v>46160.65298813657</v>
+        <v>46160.81215837963</v>
       </c>
       <c r="C121" s="9"/>
       <c r="D121" s="8">
-        <v>46217.16837645833</v>
+        <v>46217.168417002315</v>
       </c>
       <c r="E121" s="9" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>26</v>
@@ -8791,13 +8794,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="O121" s="9" t="s">
-        <v>216</v>
+        <v>334</v>
       </c>
       <c r="P121" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="Q121" s="9"/>
       <c r="R121" s="9"/>
@@ -8810,11 +8813,11 @@
         <v>364</v>
       </c>
       <c r="B122" s="5">
-        <v>46160.81215837963</v>
+        <v>46160.81220768519</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46217.168417002315</v>
+        <v>46217.16841864583</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>334</v>
@@ -8844,13 +8847,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>334</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8863,30 +8866,24 @@
         <v>365</v>
       </c>
       <c r="B123" s="8">
-        <v>46160.81220768519</v>
+        <v>46160.65302554399</v>
       </c>
       <c r="C123" s="9"/>
       <c r="D123" s="8">
-        <v>46217.16841864583</v>
+        <v>46160.8192895949</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>334</v>
+        <v>366</v>
       </c>
       <c r="F123" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G123" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="H123" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="I123" s="8">
-        <v>46217</v>
-      </c>
-      <c r="J123" s="8">
-        <v>46217</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H123" s="9"/>
+      <c r="I123" s="9"/>
+      <c r="J123" s="9"/>
       <c r="K123" s="9" t="s">
         <v>26</v>
       </c>
@@ -8894,16 +8891,16 @@
         <v>26</v>
       </c>
       <c r="M123" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>360</v>
+        <v>26</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>334</v>
+        <v>367</v>
       </c>
       <c r="P123" s="9" t="s">
-        <v>360</v>
+        <v>26</v>
       </c>
       <c r="Q123" s="9"/>
       <c r="R123" s="9"/>
@@ -8913,27 +8910,33 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B124" s="5">
-        <v>46160.65302554399</v>
+        <v>46160.65302895833</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46160.8192895949</v>
+        <v>46219.173083553236</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H124" s="6"/>
-      <c r="I124" s="6"/>
-      <c r="J124" s="6"/>
+        <v>370</v>
+      </c>
+      <c r="H124" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="I124" s="5">
+        <v>46218</v>
+      </c>
+      <c r="J124" s="5">
+        <v>46226</v>
+      </c>
       <c r="K124" s="6" t="s">
         <v>26</v>
       </c>
@@ -8941,45 +8944,55 @@
         <v>26</v>
       </c>
       <c r="M124" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N124" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="O124" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="P124" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="Q124" s="5">
+        <v>46218</v>
+      </c>
+      <c r="R124" s="5">
+        <v>46226</v>
+      </c>
+      <c r="S124" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="T124" s="6">
         <v>0</v>
       </c>
-      <c r="N124" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O124" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="P124" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q124" s="6"/>
-      <c r="R124" s="6"/>
-      <c r="S124" s="6"/>
-      <c r="T124" s="6"/>
-      <c r="U124" s="6"/>
+      <c r="U124" s="11" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="B125" s="8">
-        <v>46160.65302895833</v>
+        <v>46160.65303386574</v>
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="8">
-        <v>46219.173083553236</v>
+        <v>46219.17308424768</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>371</v>
+        <v>36</v>
       </c>
       <c r="H125" s="9" t="s">
-        <v>372</v>
+        <v>37</v>
       </c>
       <c r="I125" s="8">
         <v>46218</v>
@@ -8997,13 +9010,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="O125" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="P125" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="Q125" s="8">
         <v>46218</v>
@@ -9012,7 +9025,7 @@
         <v>46226</v>
       </c>
       <c r="S125" s="12" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="T125" s="9">
         <v>0</v>
@@ -9023,33 +9036,27 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B126" s="5">
-        <v>46160.65303386574</v>
+        <v>46160.65808951389</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46219.17308424768</v>
+        <v>46160.819809513894</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H126" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I126" s="5">
-        <v>46218</v>
-      </c>
-      <c r="J126" s="5">
-        <v>46226</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H126" s="6"/>
+      <c r="I126" s="6"/>
+      <c r="J126" s="6"/>
       <c r="K126" s="6" t="s">
         <v>26</v>
       </c>
@@ -9057,25 +9064,21 @@
         <v>26</v>
       </c>
       <c r="M126" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>367</v>
+        <v>26</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>360</v>
+        <v>377</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>367</v>
-      </c>
-      <c r="Q126" s="5">
-        <v>46218</v>
-      </c>
-      <c r="R126" s="5">
-        <v>46226</v>
-      </c>
-      <c r="S126" s="12" t="s">
-        <v>373</v>
+        <v>26</v>
+      </c>
+      <c r="Q126" s="6"/>
+      <c r="R126" s="6"/>
+      <c r="S126" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T126" s="6">
         <v>0</v>
@@ -9086,27 +9089,33 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B127" s="8">
-        <v>46160.65808951389</v>
+        <v>46160.66095159722</v>
       </c>
       <c r="C127" s="9"/>
       <c r="D127" s="8">
-        <v>46160.819809513894</v>
+        <v>46219.173089097225</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F127" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G127" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H127" s="9"/>
-      <c r="I127" s="9"/>
-      <c r="J127" s="9"/>
+        <v>54</v>
+      </c>
+      <c r="H127" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="I127" s="8">
+        <v>46218</v>
+      </c>
+      <c r="J127" s="8">
+        <v>46226</v>
+      </c>
       <c r="K127" s="9" t="s">
         <v>26</v>
       </c>
@@ -9114,21 +9123,25 @@
         <v>26</v>
       </c>
       <c r="M127" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>26</v>
+        <v>376</v>
       </c>
       <c r="O127" s="9" t="s">
-        <v>378</v>
+        <v>359</v>
       </c>
       <c r="P127" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q127" s="9"/>
-      <c r="R127" s="9"/>
-      <c r="S127" s="10" t="s">
-        <v>32</v>
+        <v>380</v>
+      </c>
+      <c r="Q127" s="8">
+        <v>46218</v>
+      </c>
+      <c r="R127" s="8">
+        <v>46226</v>
+      </c>
+      <c r="S127" s="12" t="s">
+        <v>372</v>
       </c>
       <c r="T127" s="9">
         <v>0</v>
@@ -9139,17 +9152,17 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B128" s="5">
-        <v>46160.66095159722</v>
+        <v>46160.66107538194</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46219.173089097225</v>
+        <v>46160.8199466088</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
@@ -9161,10 +9174,10 @@
         <v>55</v>
       </c>
       <c r="I128" s="5">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="J128" s="5">
-        <v>46226</v>
+        <v>46237</v>
       </c>
       <c r="K128" s="6" t="s">
         <v>26</v>
@@ -9176,90 +9189,27 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="Q128" s="5">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="R128" s="5">
-        <v>46226</v>
-      </c>
-      <c r="S128" s="12" t="s">
-        <v>373</v>
+        <v>46237</v>
+      </c>
+      <c r="S128" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T128" s="6">
         <v>0</v>
       </c>
       <c r="U128" s="11" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A129" s="7" t="s">
-        <v>382</v>
-      </c>
-      <c r="B129" s="8">
-        <v>46160.66107538194</v>
-      </c>
-      <c r="C129" s="9"/>
-      <c r="D129" s="8">
-        <v>46160.8199466088</v>
-      </c>
-      <c r="E129" s="9" t="s">
-        <v>383</v>
-      </c>
-      <c r="F129" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G129" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="H129" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I129" s="8">
-        <v>46227</v>
-      </c>
-      <c r="J129" s="8">
-        <v>46237</v>
-      </c>
-      <c r="K129" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L129" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M129" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N129" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="O129" s="9" t="s">
-        <v>380</v>
-      </c>
-      <c r="P129" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="Q129" s="8">
-        <v>46227</v>
-      </c>
-      <c r="R129" s="8">
-        <v>46237</v>
-      </c>
-      <c r="S129" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="T129" s="9">
-        <v>0</v>
-      </c>
-      <c r="U129" s="11" t="s">
         <v>120</v>
       </c>
     </row>

</xml_diff>